<commit_message>
exclude particular articles feature
</commit_message>
<xml_diff>
--- a/data/mapping.xlsx
+++ b/data/mapping.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\web\Node\parse-fabric-stocks\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23256" windowHeight="13176"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23250" windowHeight="13170" firstSheet="1" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="GT_Byaz_220_120" sheetId="1" r:id="rId1"/>
@@ -9472,7 +9477,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="8">
     <font>
       <sz val="11"/>
@@ -9642,7 +9647,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -9966,7 +9971,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -9974,15 +9979,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C216"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <dimension ref="A1:D216"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="24.3984375" customWidth="1"/>
-    <col min="2" max="2" width="48.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.375" customWidth="1"/>
+    <col min="2" max="2" width="48.75" customWidth="1"/>
     <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -9992,8 +9997,11 @@
       <c r="C1" s="2" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -10003,8 +10011,11 @@
       <c r="C2" s="2" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -10015,7 +10026,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -10026,7 +10037,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -10037,7 +10048,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -10048,7 +10059,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:4">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -10059,7 +10070,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:4">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -10070,7 +10081,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:4">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -10081,7 +10092,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:4">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -10092,7 +10103,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:4">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -10103,7 +10114,7 @@
         <v>2044186087804</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:4">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -10114,7 +10125,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:4">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -10125,7 +10136,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:4">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -10136,7 +10147,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:4">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -10147,7 +10158,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:4">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -12299,10 +12310,10 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="20.8984375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="20.875" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -12650,11 +12661,11 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C108"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="40.5" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="20.09765625" customWidth="1"/>
+    <col min="3" max="3" width="20.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15">
@@ -13854,11 +13865,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C26"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="27.19921875" customWidth="1"/>
-    <col min="2" max="2" width="51.3984375" customWidth="1"/>
-    <col min="3" max="3" width="16.3984375" customWidth="1"/>
+    <col min="1" max="1" width="27.25" customWidth="1"/>
+    <col min="2" max="2" width="51.375" customWidth="1"/>
+    <col min="3" max="3" width="16.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -14155,11 +14166,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C140"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="23.3984375" customWidth="1"/>
-    <col min="2" max="2" width="47.59765625" customWidth="1"/>
-    <col min="3" max="3" width="16.19921875" customWidth="1"/>
+    <col min="1" max="1" width="23.375" customWidth="1"/>
+    <col min="2" max="2" width="47.625" customWidth="1"/>
+    <col min="3" max="3" width="16.25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -15707,10 +15718,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C71"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="21.59765625" customWidth="1"/>
-    <col min="2" max="2" width="49.8984375" customWidth="1"/>
+    <col min="1" max="1" width="21.625" customWidth="1"/>
+    <col min="2" max="2" width="49.875" customWidth="1"/>
     <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -16504,10 +16515,10 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="27.8984375" customWidth="1"/>
-    <col min="2" max="2" width="37.296875" customWidth="1"/>
+    <col min="1" max="1" width="27.875" customWidth="1"/>
+    <col min="2" max="2" width="37.25" customWidth="1"/>
     <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -16761,9 +16772,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="25.09765625" customWidth="1"/>
+    <col min="1" max="1" width="25.125" customWidth="1"/>
     <col min="5" max="5" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -17017,11 +17028,11 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C216"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="31.8984375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="46.3984375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="14.8984375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="31.875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="46.375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="14.875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -18501,15 +18512,15 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C691"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <dimension ref="A1:D691"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="30.3984375" customWidth="1"/>
-    <col min="2" max="2" width="14.3984375" customWidth="1"/>
-    <col min="3" max="3" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.375" customWidth="1"/>
+    <col min="2" max="2" width="14.375" customWidth="1"/>
+    <col min="3" max="3" width="16.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>524</v>
       </c>
@@ -18519,8 +18530,11 @@
       <c r="C1" t="s">
         <v>786</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>525</v>
       </c>
@@ -18531,7 +18545,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>526</v>
       </c>
@@ -18542,7 +18556,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>527</v>
       </c>
@@ -18553,7 +18567,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>528</v>
       </c>
@@ -18564,7 +18578,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>529</v>
       </c>
@@ -18575,7 +18589,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>530</v>
       </c>
@@ -18586,7 +18600,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>531</v>
       </c>
@@ -18597,7 +18611,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>532</v>
       </c>
@@ -18608,7 +18622,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>533</v>
       </c>
@@ -18619,7 +18633,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>534</v>
       </c>
@@ -18630,7 +18644,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>535</v>
       </c>
@@ -18641,7 +18655,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>536</v>
       </c>
@@ -18652,7 +18666,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>537</v>
       </c>
@@ -18663,7 +18677,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:4">
       <c r="A15" t="s">
         <v>538</v>
       </c>
@@ -18674,7 +18688,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>539</v>
       </c>
@@ -23033,7 +23047,7 @@
         <v>2047878477921</v>
       </c>
     </row>
-    <row r="423" spans="1:3" ht="14.4" thickBot="1">
+    <row r="423" spans="1:3" ht="15" thickBot="1">
       <c r="A423" s="10" t="s">
         <v>2385</v>
       </c>
@@ -23042,7 +23056,7 @@
         <v>2047878477938</v>
       </c>
     </row>
-    <row r="424" spans="1:3" ht="14.4" thickBot="1">
+    <row r="424" spans="1:3" ht="15" thickBot="1">
       <c r="A424" s="10" t="s">
         <v>2386</v>
       </c>
@@ -23053,7 +23067,7 @@
         <v>2047878477952</v>
       </c>
     </row>
-    <row r="425" spans="1:3" ht="14.4" thickBot="1">
+    <row r="425" spans="1:3" ht="15" thickBot="1">
       <c r="A425" s="10" t="s">
         <v>2387</v>
       </c>
@@ -23064,7 +23078,7 @@
         <v>2047878477976</v>
       </c>
     </row>
-    <row r="426" spans="1:3" ht="14.4" thickBot="1">
+    <row r="426" spans="1:3" ht="15" thickBot="1">
       <c r="A426" s="10" t="s">
         <v>2388</v>
       </c>
@@ -23565,7 +23579,7 @@
         <v>2047878478737</v>
       </c>
     </row>
-    <row r="474" spans="1:3" ht="14.4" thickBot="1">
+    <row r="474" spans="1:3" ht="15" thickBot="1">
       <c r="A474" t="s">
         <v>2490</v>
       </c>
@@ -23574,7 +23588,7 @@
         <v>2047878478751</v>
       </c>
     </row>
-    <row r="475" spans="1:3" ht="14.4" thickBot="1">
+    <row r="475" spans="1:3" ht="15" thickBot="1">
       <c r="A475" t="s">
         <v>2491</v>
       </c>
@@ -23656,7 +23670,7 @@
         <v>2047878478904</v>
       </c>
     </row>
-    <row r="483" spans="1:3" ht="14.4" thickBot="1">
+    <row r="483" spans="1:3" ht="15" thickBot="1">
       <c r="A483" t="s">
         <v>2499</v>
       </c>
@@ -23667,7 +23681,7 @@
         <v>2047878478911</v>
       </c>
     </row>
-    <row r="484" spans="1:3" ht="14.4" thickBot="1">
+    <row r="484" spans="1:3" ht="15" thickBot="1">
       <c r="A484" t="s">
         <v>2500</v>
       </c>
@@ -25339,7 +25353,7 @@
         <v>2047983960523</v>
       </c>
     </row>
-    <row r="642" spans="1:3" ht="14.4" thickBot="1">
+    <row r="642" spans="1:3" ht="15" thickBot="1">
       <c r="A642" s="15" t="s">
         <v>2813</v>
       </c>
@@ -25348,7 +25362,7 @@
         <v>2047983960561</v>
       </c>
     </row>
-    <row r="643" spans="1:3" ht="14.4" thickBot="1">
+    <row r="643" spans="1:3" ht="15" thickBot="1">
       <c r="A643" s="15" t="s">
         <v>2814</v>
       </c>
@@ -25780,16 +25794,16 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D153"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <dimension ref="A1:E153"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="28.69921875" customWidth="1"/>
+    <col min="1" max="1" width="28.75" customWidth="1"/>
     <col min="2" max="2" width="37" customWidth="1"/>
-    <col min="3" max="3" width="9.09765625" customWidth="1"/>
-    <col min="4" max="4" width="11.8984375" customWidth="1"/>
+    <col min="3" max="3" width="9.125" customWidth="1"/>
+    <col min="4" max="4" width="11.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="5" t="s">
         <v>1513</v>
       </c>
@@ -25802,8 +25816,11 @@
       <c r="D1">
         <v>2045411146990</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="5" t="s">
         <v>1516</v>
       </c>
@@ -25817,7 +25834,7 @@
         <v>2045411147553</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
         <v>1519</v>
       </c>
@@ -25831,7 +25848,7 @@
         <v>2045411146952</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:5">
       <c r="A4" s="5" t="s">
         <v>1522</v>
       </c>
@@ -25845,7 +25862,7 @@
         <v>2045411146860</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
         <v>1525</v>
       </c>
@@ -25859,7 +25876,7 @@
         <v>2045411147409</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:5">
       <c r="A6" s="5" t="s">
         <v>1528</v>
       </c>
@@ -25873,7 +25890,7 @@
         <v>2045411147348</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:5">
       <c r="A7" s="5" t="s">
         <v>1531</v>
       </c>
@@ -25887,7 +25904,7 @@
         <v>2045411146693</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:5">
       <c r="A8" s="5" t="s">
         <v>1534</v>
       </c>
@@ -25901,7 +25918,7 @@
         <v>2045411146969</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:5">
       <c r="A9" s="5" t="s">
         <v>1537</v>
       </c>
@@ -25915,7 +25932,7 @@
         <v>2045411146747</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:5">
       <c r="A10" s="5" t="s">
         <v>1540</v>
       </c>
@@ -25929,7 +25946,7 @@
         <v>2045411146785</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
         <v>1543</v>
       </c>
@@ -25943,7 +25960,7 @@
         <v>2045411147027</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
         <v>1546</v>
       </c>
@@ -25957,7 +25974,7 @@
         <v>2045411147263</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:5">
       <c r="A13" s="5" t="s">
         <v>1549</v>
       </c>
@@ -25971,7 +25988,7 @@
         <v>2045411146303</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:5">
       <c r="A14" s="5" t="s">
         <v>1552</v>
       </c>
@@ -25985,7 +26002,7 @@
         <v>2045411146808</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:5">
       <c r="A15" s="5" t="s">
         <v>1555</v>
       </c>
@@ -25999,7 +26016,7 @@
         <v>2045411146815</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:5">
       <c r="A16" s="5" t="s">
         <v>1558</v>
       </c>

</xml_diff>